<commit_message>
Update NG Swing GDD master prices
</commit_message>
<xml_diff>
--- a/master/master_ng_swing_gdd.xlsx
+++ b/master/master_ng_swing_gdd.xlsx
@@ -9,7 +9,7 @@
     <sheet name="NG Swing GDD" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NG Swing GDD'!$A$1:$F$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NG Swing GDD'!$A$1:$G$70</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -498,25 +499,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
@@ -529,13 +535,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
+        <v>3.035</v>
+      </c>
+      <c r="C2" s="3" t="n">
         <v>2.91</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="D2" s="3" t="n">
         <v>2.8799</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>2.9</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>2.9</v>
@@ -543,6 +549,9 @@
       <c r="F2" s="3" t="n">
         <v>2.9</v>
       </c>
+      <c r="G2" s="3" t="n">
+        <v>2.9</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -551,13 +560,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>2.61</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="D3" s="3" t="n">
         <v>2.6174</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>2.758</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>2.758</v>
@@ -565,6 +574,9 @@
       <c r="F3" s="3" t="n">
         <v>2.758</v>
       </c>
+      <c r="G3" s="3" t="n">
+        <v>2.758</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -573,13 +585,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
+        <v>2.175</v>
+      </c>
+      <c r="C4" s="3" t="n">
         <v>2.61</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="D4" s="3" t="n">
         <v>2.95</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>2.803</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>2.803</v>
@@ -587,6 +599,9 @@
       <c r="F4" s="3" t="n">
         <v>2.803</v>
       </c>
+      <c r="G4" s="3" t="n">
+        <v>2.803</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -595,13 +610,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C5" s="3" t="n">
         <v>2.78</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="D5" s="3" t="n">
         <v>2.814</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>2.826</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>2.826</v>
@@ -609,6 +624,9 @@
       <c r="F5" s="3" t="n">
         <v>2.826</v>
       </c>
+      <c r="G5" s="3" t="n">
+        <v>2.826</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -617,13 +635,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
+        <v>2.965</v>
+      </c>
+      <c r="C6" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="D6" s="3" t="n">
         <v>2.8136</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>2.795</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>2.795</v>
@@ -631,6 +649,9 @@
       <c r="F6" s="3" t="n">
         <v>2.795</v>
       </c>
+      <c r="G6" s="3" t="n">
+        <v>2.795</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -639,13 +660,13 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>2.165</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="D7" s="3" t="n">
         <v>1.935</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>1.815</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>1.815</v>
@@ -653,6 +674,9 @@
       <c r="F7" s="3" t="n">
         <v>1.815</v>
       </c>
+      <c r="G7" s="3" t="n">
+        <v>1.815</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -661,13 +685,13 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C8" s="3" t="n">
         <v>2.245</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="D8" s="3" t="n">
         <v>1.958</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>1.815</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>1.815</v>
@@ -675,6 +699,9 @@
       <c r="F8" s="3" t="n">
         <v>1.815</v>
       </c>
+      <c r="G8" s="3" t="n">
+        <v>1.815</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -683,13 +710,13 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
+        <v>2.635</v>
+      </c>
+      <c r="C9" s="3" t="n">
         <v>2.76</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="D9" s="3" t="n">
         <v>2.7246</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>2.83</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2.83</v>
@@ -697,6 +724,9 @@
       <c r="F9" s="3" t="n">
         <v>2.83</v>
       </c>
+      <c r="G9" s="3" t="n">
+        <v>2.83</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -705,13 +735,13 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
+        <v>2.575</v>
+      </c>
+      <c r="C10" s="3" t="n">
         <v>2.75</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="D10" s="3" t="n">
         <v>2.8088</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>2.78</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>2.78</v>
@@ -719,6 +749,9 @@
       <c r="F10" s="3" t="n">
         <v>2.78</v>
       </c>
+      <c r="G10" s="3" t="n">
+        <v>2.78</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -727,13 +760,13 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="C11" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="D11" s="3" t="n">
         <v>1.7466</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>1.204</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>1.204</v>
@@ -741,6 +774,9 @@
       <c r="F11" s="3" t="n">
         <v>1.204</v>
       </c>
+      <c r="G11" s="3" t="n">
+        <v>1.204</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -749,13 +785,13 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="C12" s="3" t="n">
         <v>2.425</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="D12" s="3" t="n">
         <v>2.4222</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>2.485</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>2.485</v>
@@ -763,6 +799,9 @@
       <c r="F12" s="3" t="n">
         <v>2.485</v>
       </c>
+      <c r="G12" s="3" t="n">
+        <v>2.485</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -771,13 +810,13 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="C13" s="3" t="n">
         <v>2.77</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="D13" s="3" t="n">
         <v>2.8214</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>2.832</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>2.832</v>
@@ -785,6 +824,9 @@
       <c r="F13" s="3" t="n">
         <v>2.832</v>
       </c>
+      <c r="G13" s="3" t="n">
+        <v>2.832</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -793,13 +835,13 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
+        <v>2.535</v>
+      </c>
+      <c r="C14" s="3" t="n">
         <v>2.735</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="D14" s="3" t="n">
         <v>2.805</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>2.8</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>2.8</v>
@@ -807,6 +849,9 @@
       <c r="F14" s="3" t="n">
         <v>2.8</v>
       </c>
+      <c r="G14" s="3" t="n">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -815,13 +860,13 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
+        <v>3.555</v>
+      </c>
+      <c r="C15" s="3" t="n">
         <v>4.48</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="D15" s="3" t="n">
         <v>4.5909</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>4.545</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>4.545</v>
@@ -829,6 +874,9 @@
       <c r="F15" s="3" t="n">
         <v>4.545</v>
       </c>
+      <c r="G15" s="3" t="n">
+        <v>4.545</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -837,13 +885,13 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
+        <v>2.835</v>
+      </c>
+      <c r="C16" s="3" t="n">
         <v>2.74</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="D16" s="3" t="n">
         <v>2.7991</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>2.55</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>2.55</v>
@@ -851,6 +899,9 @@
       <c r="F16" s="3" t="n">
         <v>2.55</v>
       </c>
+      <c r="G16" s="3" t="n">
+        <v>2.55</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -859,13 +910,13 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="C17" s="3" t="n">
         <v>3.215</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="D17" s="3" t="n">
         <v>3.2871</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>3.285</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>3.285</v>
@@ -873,6 +924,9 @@
       <c r="F17" s="3" t="n">
         <v>3.285</v>
       </c>
+      <c r="G17" s="3" t="n">
+        <v>3.285</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -881,13 +935,13 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="C18" s="3" t="n">
         <v>2.69</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="D18" s="3" t="n">
         <v>2.799</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>2.59</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>2.59</v>
@@ -895,6 +949,9 @@
       <c r="F18" s="3" t="n">
         <v>2.59</v>
       </c>
+      <c r="G18" s="3" t="n">
+        <v>2.59</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -903,13 +960,13 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
+        <v>2.455</v>
+      </c>
+      <c r="C19" s="3" t="n">
         <v>2.76</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="D19" s="3" t="n">
         <v>2.8072</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>2.5835</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>2.5835</v>
@@ -917,6 +974,9 @@
       <c r="F19" s="3" t="n">
         <v>2.5835</v>
       </c>
+      <c r="G19" s="3" t="n">
+        <v>2.5835</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -925,13 +985,13 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="C20" s="3" t="n">
         <v>2.745</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="D20" s="3" t="n">
         <v>2.788</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>2.5755</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>2.5755</v>
@@ -939,6 +999,9 @@
       <c r="F20" s="3" t="n">
         <v>2.5755</v>
       </c>
+      <c r="G20" s="3" t="n">
+        <v>2.5755</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -947,13 +1010,13 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C21" s="3" t="n">
         <v>2.375</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="D21" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>2.156</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>2.156</v>
@@ -961,6 +1024,9 @@
       <c r="F21" s="3" t="n">
         <v>2.156</v>
       </c>
+      <c r="G21" s="3" t="n">
+        <v>2.156</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -969,13 +1035,13 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C22" s="3" t="n">
         <v>2.75</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="D22" s="3" t="n">
         <v>2.8098</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>2.866</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>2.866</v>
@@ -983,6 +1049,9 @@
       <c r="F22" s="3" t="n">
         <v>2.866</v>
       </c>
+      <c r="G22" s="3" t="n">
+        <v>2.866</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -991,13 +1060,13 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="C23" s="3" t="n">
         <v>2.4</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="D23" s="3" t="n">
         <v>2.35</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>2.525</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>2.525</v>
@@ -1005,6 +1074,9 @@
       <c r="F23" s="3" t="n">
         <v>2.525</v>
       </c>
+      <c r="G23" s="3" t="n">
+        <v>2.525</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1013,13 +1085,13 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="C24" s="3" t="n">
         <v>2.665</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="D24" s="3" t="n">
         <v>2.6798</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>2.781</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>2.781</v>
@@ -1027,6 +1099,9 @@
       <c r="F24" s="3" t="n">
         <v>2.781</v>
       </c>
+      <c r="G24" s="3" t="n">
+        <v>2.781</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1035,13 +1110,13 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="C25" s="3" t="n">
         <v>2.715</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="D25" s="3" t="n">
         <v>2.7689</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>2.81</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>2.81</v>
@@ -1049,6 +1124,9 @@
       <c r="F25" s="3" t="n">
         <v>2.81</v>
       </c>
+      <c r="G25" s="3" t="n">
+        <v>2.81</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1057,13 +1135,13 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="C26" s="3" t="n">
         <v>2.74</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="D26" s="3" t="n">
         <v>2.7496</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>2.81</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>2.81</v>
@@ -1071,6 +1149,9 @@
       <c r="F26" s="3" t="n">
         <v>2.81</v>
       </c>
+      <c r="G26" s="3" t="n">
+        <v>2.81</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1079,13 +1160,13 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C27" s="3" t="n">
         <v>2.74</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="D27" s="3" t="n">
         <v>2.662</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>2.79</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>2.79</v>
@@ -1093,6 +1174,9 @@
       <c r="F27" s="3" t="n">
         <v>2.79</v>
       </c>
+      <c r="G27" s="3" t="n">
+        <v>2.79</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1101,13 +1185,13 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
+        <v>2.565</v>
+      </c>
+      <c r="C28" s="3" t="n">
         <v>2.73</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="D28" s="3" t="n">
         <v>2.6808</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>2.84</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>2.84</v>
@@ -1115,6 +1199,9 @@
       <c r="F28" s="3" t="n">
         <v>2.84</v>
       </c>
+      <c r="G28" s="3" t="n">
+        <v>2.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1123,13 +1210,13 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="C29" s="3" t="n">
         <v>2.245</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="D29" s="3" t="n">
         <v>2.05</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>1.99</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>1.99</v>
@@ -1137,6 +1224,9 @@
       <c r="F29" s="3" t="n">
         <v>1.99</v>
       </c>
+      <c r="G29" s="3" t="n">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1145,10 +1235,10 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C30" s="3" t="n">
         <v>1.245</v>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>1.572</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>1.572</v>
@@ -1159,6 +1249,9 @@
       <c r="F30" s="3" t="n">
         <v>1.572</v>
       </c>
+      <c r="G30" s="3" t="n">
+        <v>1.572</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1167,13 +1260,13 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
+        <v>2.655</v>
+      </c>
+      <c r="C31" s="3" t="n">
         <v>2.65</v>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="D31" s="3" t="n">
         <v>2.6526</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>2.6865</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>2.6865</v>
@@ -1181,6 +1274,9 @@
       <c r="F31" s="3" t="n">
         <v>2.6865</v>
       </c>
+      <c r="G31" s="3" t="n">
+        <v>2.6865</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1189,13 +1285,13 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="C32" s="3" t="n">
         <v>2.075</v>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="D32" s="3" t="n">
         <v>1.9591</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>1.99</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>1.99</v>
@@ -1203,6 +1299,9 @@
       <c r="F32" s="3" t="n">
         <v>1.99</v>
       </c>
+      <c r="G32" s="3" t="n">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1211,13 +1310,13 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
+        <v>1.495</v>
+      </c>
+      <c r="C33" s="3" t="n">
         <v>1.41</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="D33" s="3" t="n">
         <v>1.3192</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>1.34</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>1.34</v>
@@ -1225,6 +1324,9 @@
       <c r="F33" s="3" t="n">
         <v>1.34</v>
       </c>
+      <c r="G33" s="3" t="n">
+        <v>1.34</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1233,13 +1335,13 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C34" s="3" t="n">
         <v>2.64</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="D34" s="3" t="n">
         <v>2.6338</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>2.71</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>2.71</v>
@@ -1247,6 +1349,9 @@
       <c r="F34" s="3" t="n">
         <v>2.71</v>
       </c>
+      <c r="G34" s="3" t="n">
+        <v>2.71</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1255,13 +1360,13 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="C35" s="3" t="n">
         <v>1.51</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="D35" s="3" t="n">
         <v>1.7958</v>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>1.38</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>1.38</v>
@@ -1269,6 +1374,9 @@
       <c r="F35" s="3" t="n">
         <v>1.38</v>
       </c>
+      <c r="G35" s="3" t="n">
+        <v>1.38</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1277,13 +1385,13 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="C36" s="3" t="n">
         <v>2.93</v>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="D36" s="3" t="n">
         <v>2.9677</v>
-      </c>
-      <c r="D36" s="3" t="n">
-        <v>2.992</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>2.992</v>
@@ -1291,6 +1399,9 @@
       <c r="F36" s="3" t="n">
         <v>2.992</v>
       </c>
+      <c r="G36" s="3" t="n">
+        <v>2.992</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1299,13 +1410,13 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
+        <v>2.605</v>
+      </c>
+      <c r="C37" s="3" t="n">
         <v>2.725</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="D37" s="3" t="n">
         <v>2.7289</v>
-      </c>
-      <c r="D37" s="3" t="n">
-        <v>2.785</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>2.785</v>
@@ -1313,6 +1424,9 @@
       <c r="F37" s="3" t="n">
         <v>2.785</v>
       </c>
+      <c r="G37" s="3" t="n">
+        <v>2.785</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1321,13 +1435,13 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C38" s="3" t="n">
         <v>2.255</v>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="D38" s="3" t="n">
         <v>2.007</v>
-      </c>
-      <c r="D38" s="3" t="n">
-        <v>2.135</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>2.135</v>
@@ -1335,6 +1449,9 @@
       <c r="F38" s="3" t="n">
         <v>2.135</v>
       </c>
+      <c r="G38" s="3" t="n">
+        <v>2.135</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1343,13 +1460,13 @@
         </is>
       </c>
       <c r="B39" s="3" t="n">
+        <v>1.415</v>
+      </c>
+      <c r="C39" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="D39" s="3" t="n">
         <v>2.5482</v>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>2.485</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>2.485</v>
@@ -1357,6 +1474,9 @@
       <c r="F39" s="3" t="n">
         <v>2.485</v>
       </c>
+      <c r="G39" s="3" t="n">
+        <v>2.485</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1365,13 +1485,13 @@
         </is>
       </c>
       <c r="B40" s="3" t="n">
+        <v>2.505</v>
+      </c>
+      <c r="C40" s="3" t="n">
         <v>3.29</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="D40" s="3" t="n">
         <v>3.2201</v>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>3.375</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>3.375</v>
@@ -1379,6 +1499,9 @@
       <c r="F40" s="3" t="n">
         <v>3.375</v>
       </c>
+      <c r="G40" s="3" t="n">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1387,13 +1510,13 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="C41" s="3" t="n">
         <v>4.315</v>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="D41" s="3" t="n">
         <v>4.4174</v>
-      </c>
-      <c r="D41" s="3" t="n">
-        <v>4.363</v>
       </c>
       <c r="E41" s="3" t="n">
         <v>4.363</v>
@@ -1401,6 +1524,9 @@
       <c r="F41" s="3" t="n">
         <v>4.363</v>
       </c>
+      <c r="G41" s="3" t="n">
+        <v>4.363</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1409,13 +1535,13 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
+        <v>2.545</v>
+      </c>
+      <c r="C42" s="3" t="n">
         <v>2.615</v>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="D42" s="3" t="n">
         <v>2.6647</v>
-      </c>
-      <c r="D42" s="3" t="n">
-        <v>2.71</v>
       </c>
       <c r="E42" s="3" t="n">
         <v>2.71</v>
@@ -1423,6 +1549,9 @@
       <c r="F42" s="3" t="n">
         <v>2.71</v>
       </c>
+      <c r="G42" s="3" t="n">
+        <v>2.71</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1431,13 +1560,13 @@
         </is>
       </c>
       <c r="B43" s="3" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="C43" s="3" t="n">
         <v>2.56</v>
       </c>
-      <c r="C43" s="3" t="n">
+      <c r="D43" s="3" t="n">
         <v>2.5612</v>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>2.6805</v>
       </c>
       <c r="E43" s="3" t="n">
         <v>2.6805</v>
@@ -1445,6 +1574,9 @@
       <c r="F43" s="3" t="n">
         <v>2.6805</v>
       </c>
+      <c r="G43" s="3" t="n">
+        <v>2.6805</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1453,13 +1585,13 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="C44" s="3" t="n">
         <v>2.915</v>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="D44" s="3" t="n">
         <v>2.9</v>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>3.042</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>3.042</v>
@@ -1467,6 +1599,9 @@
       <c r="F44" s="3" t="n">
         <v>3.042</v>
       </c>
+      <c r="G44" s="3" t="n">
+        <v>3.042</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1475,13 +1610,13 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
+        <v>2.045</v>
+      </c>
+      <c r="C45" s="3" t="n">
         <v>2.42</v>
       </c>
-      <c r="C45" s="3" t="n">
+      <c r="D45" s="3" t="n">
         <v>2.4175</v>
-      </c>
-      <c r="D45" s="3" t="n">
-        <v>2.475</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>2.475</v>
@@ -1489,6 +1624,9 @@
       <c r="F45" s="3" t="n">
         <v>2.475</v>
       </c>
+      <c r="G45" s="3" t="n">
+        <v>2.475</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1497,13 +1635,13 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="C46" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="D46" s="3" t="n">
         <v>2.4926</v>
-      </c>
-      <c r="D46" s="3" t="n">
-        <v>2.48</v>
       </c>
       <c r="E46" s="3" t="n">
         <v>2.48</v>
@@ -1511,6 +1649,9 @@
       <c r="F46" s="3" t="n">
         <v>2.48</v>
       </c>
+      <c r="G46" s="3" t="n">
+        <v>2.48</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1519,13 +1660,13 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
+        <v>2.835</v>
+      </c>
+      <c r="C47" s="3" t="n">
         <v>2.72</v>
       </c>
-      <c r="C47" s="3" t="n">
+      <c r="D47" s="3" t="n">
         <v>2.7743</v>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>2.786</v>
       </c>
       <c r="E47" s="3" t="n">
         <v>2.786</v>
@@ -1533,6 +1674,9 @@
       <c r="F47" s="3" t="n">
         <v>2.786</v>
       </c>
+      <c r="G47" s="3" t="n">
+        <v>2.786</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1541,13 +1685,13 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="C48" s="3" t="n">
         <v>2.905</v>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="D48" s="3" t="n">
         <v>2.9772</v>
-      </c>
-      <c r="D48" s="3" t="n">
-        <v>2.992</v>
       </c>
       <c r="E48" s="3" t="n">
         <v>2.992</v>
@@ -1555,6 +1699,9 @@
       <c r="F48" s="3" t="n">
         <v>2.992</v>
       </c>
+      <c r="G48" s="3" t="n">
+        <v>2.992</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1563,13 +1710,13 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="C49" s="3" t="n">
         <v>4.295</v>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="D49" s="3" t="n">
         <v>4.3206</v>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>4.245</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>4.245</v>
@@ -1577,6 +1724,9 @@
       <c r="F49" s="3" t="n">
         <v>4.245</v>
       </c>
+      <c r="G49" s="3" t="n">
+        <v>4.245</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1585,13 +1735,13 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
+        <v>2.845</v>
+      </c>
+      <c r="C50" s="3" t="n">
         <v>2.795</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="D50" s="3" t="n">
         <v>2.8</v>
-      </c>
-      <c r="D50" s="3" t="n">
-        <v>2.932</v>
       </c>
       <c r="E50" s="3" t="n">
         <v>2.932</v>
@@ -1599,6 +1749,9 @@
       <c r="F50" s="3" t="n">
         <v>2.932</v>
       </c>
+      <c r="G50" s="3" t="n">
+        <v>2.932</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1607,13 +1760,13 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="C51" s="3" t="n">
         <v>2.715</v>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="D51" s="3" t="n">
         <v>2.768</v>
-      </c>
-      <c r="D51" s="3" t="n">
-        <v>2.79</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>2.79</v>
@@ -1621,6 +1774,9 @@
       <c r="F51" s="3" t="n">
         <v>2.79</v>
       </c>
+      <c r="G51" s="3" t="n">
+        <v>2.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1629,10 +1785,10 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
+        <v>2.785</v>
+      </c>
+      <c r="C52" s="3" t="n">
         <v>2.76</v>
-      </c>
-      <c r="C52" s="3" t="n">
-        <v>2.932</v>
       </c>
       <c r="D52" s="3" t="n">
         <v>2.932</v>
@@ -1643,6 +1799,9 @@
       <c r="F52" s="3" t="n">
         <v>2.932</v>
       </c>
+      <c r="G52" s="3" t="n">
+        <v>2.932</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1651,13 +1810,13 @@
         </is>
       </c>
       <c r="B53" s="3" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="C53" s="3" t="n">
         <v>2.54</v>
       </c>
-      <c r="C53" s="3" t="n">
+      <c r="D53" s="3" t="n">
         <v>2.5115</v>
-      </c>
-      <c r="D53" s="3" t="n">
-        <v>2.685</v>
       </c>
       <c r="E53" s="3" t="n">
         <v>2.685</v>
@@ -1665,6 +1824,9 @@
       <c r="F53" s="3" t="n">
         <v>2.685</v>
       </c>
+      <c r="G53" s="3" t="n">
+        <v>2.685</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1673,13 +1835,13 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
+        <v>1.875</v>
+      </c>
+      <c r="C54" s="3" t="n">
         <v>2.405</v>
       </c>
-      <c r="C54" s="3" t="n">
+      <c r="D54" s="3" t="n">
         <v>2.3724</v>
-      </c>
-      <c r="D54" s="3" t="n">
-        <v>2.4125</v>
       </c>
       <c r="E54" s="3" t="n">
         <v>2.4125</v>
@@ -1687,6 +1849,9 @@
       <c r="F54" s="3" t="n">
         <v>2.4125</v>
       </c>
+      <c r="G54" s="3" t="n">
+        <v>2.4125</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1695,13 +1860,13 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
+        <v>2.365</v>
+      </c>
+      <c r="C55" s="3" t="n">
         <v>2.65</v>
       </c>
-      <c r="C55" s="3" t="n">
+      <c r="D55" s="3" t="n">
         <v>3.15</v>
-      </c>
-      <c r="D55" s="3" t="n">
-        <v>2.6755</v>
       </c>
       <c r="E55" s="3" t="n">
         <v>2.6755</v>
@@ -1709,6 +1874,9 @@
       <c r="F55" s="3" t="n">
         <v>2.6755</v>
       </c>
+      <c r="G55" s="3" t="n">
+        <v>2.6755</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1717,13 +1885,13 @@
         </is>
       </c>
       <c r="B56" s="3" t="n">
+        <v>2.185</v>
+      </c>
+      <c r="C56" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="C56" s="3" t="n">
+      <c r="D56" s="3" t="n">
         <v>2.95</v>
-      </c>
-      <c r="D56" s="3" t="n">
-        <v>2.581</v>
       </c>
       <c r="E56" s="3" t="n">
         <v>2.581</v>
@@ -1731,6 +1899,9 @@
       <c r="F56" s="3" t="n">
         <v>2.581</v>
       </c>
+      <c r="G56" s="3" t="n">
+        <v>2.581</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1739,13 +1910,13 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C57" s="3" t="n">
         <v>2.825</v>
       </c>
-      <c r="C57" s="3" t="n">
+      <c r="D57" s="3" t="n">
         <v>2.8203</v>
-      </c>
-      <c r="D57" s="3" t="n">
-        <v>2.934</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>2.934</v>
@@ -1753,6 +1924,9 @@
       <c r="F57" s="3" t="n">
         <v>2.934</v>
       </c>
+      <c r="G57" s="3" t="n">
+        <v>2.934</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1761,13 +1935,13 @@
         </is>
       </c>
       <c r="B58" s="3" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="C58" s="3" t="n">
         <v>2.525</v>
       </c>
-      <c r="C58" s="3" t="n">
+      <c r="D58" s="3" t="n">
         <v>2.4926</v>
-      </c>
-      <c r="D58" s="3" t="n">
-        <v>2.36</v>
       </c>
       <c r="E58" s="3" t="n">
         <v>2.36</v>
@@ -1775,6 +1949,9 @@
       <c r="F58" s="3" t="n">
         <v>2.36</v>
       </c>
+      <c r="G58" s="3" t="n">
+        <v>2.36</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1783,13 +1960,13 @@
         </is>
       </c>
       <c r="B59" s="3" t="n">
+        <v>2.755</v>
+      </c>
+      <c r="C59" s="3" t="n">
         <v>2.71</v>
       </c>
-      <c r="C59" s="3" t="n">
+      <c r="D59" s="3" t="n">
         <v>2.83</v>
-      </c>
-      <c r="D59" s="3" t="n">
-        <v>2.766</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>2.766</v>
@@ -1797,6 +1974,9 @@
       <c r="F59" s="3" t="n">
         <v>2.766</v>
       </c>
+      <c r="G59" s="3" t="n">
+        <v>2.766</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1805,13 +1985,13 @@
         </is>
       </c>
       <c r="B60" s="3" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="C60" s="3" t="n">
         <v>2.835</v>
       </c>
-      <c r="C60" s="3" t="n">
+      <c r="D60" s="3" t="n">
         <v>2.8382</v>
-      </c>
-      <c r="D60" s="3" t="n">
-        <v>3.0545</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>3.0545</v>
@@ -1819,6 +1999,9 @@
       <c r="F60" s="3" t="n">
         <v>3.0545</v>
       </c>
+      <c r="G60" s="3" t="n">
+        <v>3.0545</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1827,13 +2010,13 @@
         </is>
       </c>
       <c r="B61" s="3" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="C61" s="3" t="n">
         <v>4.275</v>
       </c>
-      <c r="C61" s="3" t="n">
+      <c r="D61" s="3" t="n">
         <v>4.3798</v>
-      </c>
-      <c r="D61" s="3" t="n">
-        <v>3.95</v>
       </c>
       <c r="E61" s="3" t="n">
         <v>3.95</v>
@@ -1841,6 +2024,9 @@
       <c r="F61" s="3" t="n">
         <v>3.95</v>
       </c>
+      <c r="G61" s="3" t="n">
+        <v>3.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1849,13 +2035,13 @@
         </is>
       </c>
       <c r="B62" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C62" s="3" t="n">
         <v>4.33</v>
       </c>
-      <c r="C62" s="3" t="n">
+      <c r="D62" s="3" t="n">
         <v>4.4409</v>
-      </c>
-      <c r="D62" s="3" t="n">
-        <v>4.685</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>4.685</v>
@@ -1863,6 +2049,9 @@
       <c r="F62" s="3" t="n">
         <v>4.685</v>
       </c>
+      <c r="G62" s="3" t="n">
+        <v>4.685</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1871,13 +2060,13 @@
         </is>
       </c>
       <c r="B63" s="3" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="C63" s="3" t="n">
         <v>2.485</v>
       </c>
-      <c r="C63" s="3" t="n">
+      <c r="D63" s="3" t="n">
         <v>2.4509</v>
-      </c>
-      <c r="D63" s="3" t="n">
-        <v>2.571</v>
       </c>
       <c r="E63" s="3" t="n">
         <v>2.571</v>
@@ -1885,6 +2074,9 @@
       <c r="F63" s="3" t="n">
         <v>2.571</v>
       </c>
+      <c r="G63" s="3" t="n">
+        <v>2.571</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1893,13 +2085,13 @@
         </is>
       </c>
       <c r="B64" s="3" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="C64" s="3" t="n">
         <v>3.555</v>
       </c>
-      <c r="C64" s="3" t="n">
+      <c r="D64" s="3" t="n">
         <v>4.4409</v>
-      </c>
-      <c r="D64" s="3" t="n">
-        <v>3.975</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>3.975</v>
@@ -1907,6 +2099,9 @@
       <c r="F64" s="3" t="n">
         <v>3.975</v>
       </c>
+      <c r="G64" s="3" t="n">
+        <v>3.975</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1915,13 +2110,13 @@
         </is>
       </c>
       <c r="B65" s="3" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="C65" s="3" t="n">
         <v>3.78</v>
       </c>
-      <c r="C65" s="3" t="n">
+      <c r="D65" s="3" t="n">
         <v>4.4485</v>
-      </c>
-      <c r="D65" s="3" t="n">
-        <v>4.346</v>
       </c>
       <c r="E65" s="3" t="n">
         <v>4.346</v>
@@ -1929,6 +2124,9 @@
       <c r="F65" s="3" t="n">
         <v>4.346</v>
       </c>
+      <c r="G65" s="3" t="n">
+        <v>4.346</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1937,13 +2135,13 @@
         </is>
       </c>
       <c r="B66" s="3" t="n">
+        <v>3.425</v>
+      </c>
+      <c r="C66" s="3" t="n">
         <v>4.36</v>
       </c>
-      <c r="C66" s="3" t="n">
+      <c r="D66" s="3" t="n">
         <v>4.4485</v>
-      </c>
-      <c r="D66" s="3" t="n">
-        <v>4.577</v>
       </c>
       <c r="E66" s="3" t="n">
         <v>4.577</v>
@@ -1951,6 +2149,9 @@
       <c r="F66" s="3" t="n">
         <v>4.577</v>
       </c>
+      <c r="G66" s="3" t="n">
+        <v>4.577</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1959,13 +2160,13 @@
         </is>
       </c>
       <c r="B67" s="3" t="n">
+        <v>2.075</v>
+      </c>
+      <c r="C67" s="3" t="n">
         <v>2.49</v>
       </c>
-      <c r="C67" s="3" t="n">
+      <c r="D67" s="3" t="n">
         <v>2.4426</v>
-      </c>
-      <c r="D67" s="3" t="n">
-        <v>2.4315</v>
       </c>
       <c r="E67" s="3" t="n">
         <v>2.4315</v>
@@ -1973,6 +2174,9 @@
       <c r="F67" s="3" t="n">
         <v>2.4315</v>
       </c>
+      <c r="G67" s="3" t="n">
+        <v>2.4315</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1981,13 +2185,13 @@
         </is>
       </c>
       <c r="B68" s="3" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="C68" s="3" t="n">
         <v>2.525</v>
       </c>
-      <c r="C68" s="3" t="n">
+      <c r="D68" s="3" t="n">
         <v>2.5</v>
-      </c>
-      <c r="D68" s="3" t="n">
-        <v>2.484</v>
       </c>
       <c r="E68" s="3" t="n">
         <v>2.484</v>
@@ -1995,6 +2199,9 @@
       <c r="F68" s="3" t="n">
         <v>2.484</v>
       </c>
+      <c r="G68" s="3" t="n">
+        <v>2.484</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2003,13 +2210,13 @@
         </is>
       </c>
       <c r="B69" s="3" t="n">
+        <v>2.745</v>
+      </c>
+      <c r="C69" s="3" t="n">
         <v>2.77</v>
       </c>
-      <c r="C69" s="3" t="n">
+      <c r="D69" s="3" t="n">
         <v>2.8253</v>
-      </c>
-      <c r="D69" s="3" t="n">
-        <v>2.892</v>
       </c>
       <c r="E69" s="3" t="n">
         <v>2.892</v>
@@ -2017,6 +2224,9 @@
       <c r="F69" s="3" t="n">
         <v>2.892</v>
       </c>
+      <c r="G69" s="3" t="n">
+        <v>2.892</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2025,13 +2235,13 @@
         </is>
       </c>
       <c r="B70" s="3" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="C70" s="3" t="n">
         <v>1.495</v>
       </c>
-      <c r="C70" s="3" t="n">
+      <c r="D70" s="3" t="n">
         <v>1.8123</v>
-      </c>
-      <c r="D70" s="3" t="n">
-        <v>1.38</v>
       </c>
       <c r="E70" s="3" t="n">
         <v>1.38</v>
@@ -2039,9 +2249,12 @@
       <c r="F70" s="3" t="n">
         <v>1.38</v>
       </c>
+      <c r="G70" s="3" t="n">
+        <v>1.38</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F70"/>
+  <autoFilter ref="A1:G70"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>